<commit_message>
feat: web en varias páginas por unidad y estadística descriptiva en R publicada
- / (inicio), /descriptiva/, /datos/, /equipo/ con estilo y JS compartidos en docs/assets
- R exporta PNG a docs/img/r y tablas CSV a docs/data/tdf para la página descriptiva
- resumen.json sin el histograma de SiO2 con la agrupación vieja
- AGENTS, README y wiki actualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R/salidas/TDF_continuas.xlsx
+++ b/R/salidas/TDF_continuas.xlsx
@@ -67,55 +67,55 @@
     <t xml:space="preserve">Hi_dsc</t>
   </si>
   <si>
-    <t xml:space="preserve">[  0.001-  5.819[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[  5.819- 11.636[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 11.636- 17.454[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 17.454- 23.271[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 23.271- 29.089[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 29.089- 34.907[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 34.907- 40.724[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 40.724- 46.542[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 46.542- 52.359[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 52.359- 58.177[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 58.177- 63.995[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 63.995- 69.812[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 69.812-  75.63[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[  75.63- 81.447[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 81.447- 87.265[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 87.265- 93.082[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 93.082-   98.9[</t>
+    <t xml:space="preserve">[0.001-5.819[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[5.819-11.636[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[11.636-17.454[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[17.454-23.271[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[23.271-29.089[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[29.089-34.907[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[34.907-40.724[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[40.724-46.542[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[46.542-52.359[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[52.359-58.177[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[58.177-63.995[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[63.995-69.812[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[69.812-75.63[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[75.63-81.447[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[81.447-87.265[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[87.265-93.082[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[93.082-98.9[</t>
   </si>
   <si>
     <t xml:space="preserve">Outliers IQR: 8413 de 57031 (14.8 %), por tipo de roca</t>
@@ -190,55 +190,55 @@
     <t xml:space="preserve">TDF corregida, toda la muestra (wt%): rango IQR + clases abiertas</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;      36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     36-     38[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     38-     40[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     40-     42[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     42-     44[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     44-     46[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     46-     48[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     48-     50[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     50-     52[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     52-     54[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     54-     56[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     56-     58[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     58-     60[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     60-     62[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     62-     64[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     64-     66[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≥      66</t>
+    <t xml:space="preserve">&lt; 36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[36-38[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[38-40[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[40-42[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[42-44[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[44-46[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[46-48[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[48-50[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[50-52[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[52-54[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[54-56[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[56-58[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[58-60[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[60-62[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[62-64[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[64-66[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 66</t>
   </si>
   <si>
     <t xml:space="preserve">Error de agrupación (toda la muestra, clases cerradas)</t>
@@ -265,43 +265,43 @@
     <t xml:space="preserve">TDF corregida, rocas volcánicas máficas (wt%)</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;      44</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     44-     45[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     45-     46[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     46-     47[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     47-     48[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     48-     49[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     49-     50[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     50-     51[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     51-     52[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     52-     53[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     53-     54[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     54-     55[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≥      55</t>
+    <t xml:space="preserve">&lt; 44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[44-45[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[45-46[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[46-47[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[47-48[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[48-49[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[49-50[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[50-51[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[51-52[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[52-53[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[53-54[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[54-55[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 55</t>
   </si>
   <si>
     <t xml:space="preserve">Error de agrupación (rocas volcánicas máficas)</t>
@@ -352,55 +352,55 @@
     <t xml:space="preserve">Curtosis</t>
   </si>
   <si>
-    <t xml:space="preserve">[0-  3.222[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[  3.222-  6.443[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[  6.443-  9.664[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[  9.664- 12.885[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 12.885- 16.106[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 16.106- 19.327[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 19.327- 22.548[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 22.548-  25.77[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[  25.77- 28.991[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 28.991- 32.212[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 32.212- 35.433[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 35.433- 38.654[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 38.654- 41.875[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 41.875- 45.097[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 45.097- 48.318[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 48.318- 51.539[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 51.539-  54.76[</t>
+    <t xml:space="preserve">[0-3.222[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[3.222-6.443[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[6.443-9.664[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[9.664-12.885[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[12.885-16.106[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[16.106-19.327[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[19.327-22.548[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[22.548-25.77[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[25.77-28.991[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[28.991-32.212[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[32.212-35.433[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[35.433-38.654[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[38.654-41.875[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[41.875-45.097[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[45.097-48.318[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[48.318-51.539[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[51.539-54.76[</t>
   </si>
   <si>
     <t xml:space="preserve">Outliers IQR: 9607 de 57039 (16.8 %), por tipo de roca</t>
@@ -412,124 +412,124 @@
     <t xml:space="preserve">vein</t>
   </si>
   <si>
-    <t xml:space="preserve">[0-      2[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      2-      4[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      4-      6[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      6-      8[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      8-     10[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     10-     12[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     12-     14[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     14-     16[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     16-     18[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     18-     20[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≥      20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;       2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      2-      3[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      3-      4[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      4-      5[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      5-      6[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      6-      7[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      7-      8[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      8-      9[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      9-     10[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     10-     11[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     11-     12[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[     12-     13[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≥      13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[  0.002-18437.5[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[18437.5-  36875[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[  36875-55312.5[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[55312.5-  73750[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[  73750-92187.5[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[92187.5- 110625[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 110625- 129063[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 129063- 147500[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 147500- 165938[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 165938- 184375[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 184375- 202813[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 202813- 221250[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 221250- 239688[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 239688- 258125[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 258125- 276563[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 276563- 295000[</t>
+    <t xml:space="preserve">[0-2[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2-4[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[4-6[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[6-8[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[8-10[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[10-12[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[12-14[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[14-16[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[16-18[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[18-20[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2-3[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[3-4[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[4-5[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[5-6[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[6-7[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[7-8[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[8-9[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[9-10[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[10-11[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[11-12[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[12-13[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.002-18437.5[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[18437.5-36875[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[36875-55312.5[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[55312.5-73750[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[73750-92187.5[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[92187.5-110625[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[110625-129063[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[129063-147500[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[147500-165938[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[165938-184375[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[184375-202813[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[202813-221250[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[221250-239688[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[239688-258125[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[258125-276563[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[276563-295000[</t>
   </si>
   <si>
     <t xml:space="preserve">Outliers IQR: 2973 de 37911 (7.8 %), por tipo de roca</t>
@@ -538,64 +538,64 @@
     <t xml:space="preserve">TDF corregida, toda la muestra (log10 ppm): rango IQR + clases abiertas</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;     0.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[    0.8-      1[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      1-    1.2[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[    1.2-    1.4[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[    1.4-    1.6[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[    1.6-    1.8[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[    1.8-      2[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      2-    2.2[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[    2.2-    2.4[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[    2.4-    2.6[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[    2.6-    2.8[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[    2.8-      3[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[      3-    3.2[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[    3.2-    3.4[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[    3.4-    3.6[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[    3.6-    3.8[</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≥     3.8</t>
+    <t xml:space="preserve">&lt; 0.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.8-1[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[1-1.2[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[1.2-1.4[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[1.4-1.6[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[1.6-1.8[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[1.8-2[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2-2.2[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2.2-2.4[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2.4-2.6[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2.6-2.8[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2.8-3[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[3-3.2[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[3.2-3.4[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[3.4-3.6[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[3.6-3.8[</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 3.8</t>
   </si>
   <si>
     <t xml:space="preserve">TDF corregida, rocas volcánicas máficas (log10 ppm)</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;     1.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≥     3.2</t>
+    <t xml:space="preserve">&lt; 1.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 3.2</t>
   </si>
   <si>
     <t xml:space="preserve">log10_toda_la_muestra</t>

</xml_diff>